<commit_message>
Add balancing targets fixture and target role to columns metadata
- ta_targets_2021.xlsx: 11 rows (trans × brch for 2021), values
  deliberately offset from actual totals to simulate balancing scenario
- columns.xlsx: add maal → target role mapping

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/fixtures/metadata/columns.xlsx
+++ b/data/fixtures/metadata/columns.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,6 +524,18 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>maal</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add BalancingConfig, TargetTolerances, Locks; rework BalancingTargets format
- BalancingTargets now mirrors SUT long-format without product dimension;
  supply uses price_basic, use uses all price columns. Removed target role
  from SUTColumns.
- Tolerances moved out of BalancingTargets into new BalancingConfig dataclass
  (field on SUT, set via set_balancing_config).
- TargetTolerances: transactions and categories DataFrames (rel/abs tolerances).
- Locks: products, transactions, categories, cells DataFrames; OR logic across
  levels. Excel sheet names match field names.
- load_balancing_config_from_excel added; metadata sub-loaders made private.
- All metadata loaders now select only specified columns, ignoring extras.
- Fixture fix: supply rows now correctly have koeb=NaN.
- New fixture: balancing_locks.xlsx.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/fixtures/metadata/columns.xlsx
+++ b/data/fixtures/metadata/columns.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,18 +524,6 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>maal</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>target</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>